<commit_message>
workaround for JAR in gitignore
</commit_message>
<xml_diff>
--- a/opentsx-clusters/mmdc-mrc/MDC-MRC.xlsx
+++ b/opentsx-clusters/mmdc-mrc/MDC-MRC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkampf/GITHUB.public/OpenTSx/opentsx-clusters/mmdc-mrc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC67F93E-FB88-3C41-9E51-2992CA5D100C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAFBC411-A5A6-7246-A7A3-68368C341ACC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3320" yWindow="1760" windowWidth="28040" windowHeight="13740" xr2:uid="{183DE6D2-7FE4-EA4F-8A21-BAAE338FD231}"/>
+    <workbookView xWindow="3320" yWindow="1760" windowWidth="28040" windowHeight="13740" activeTab="2" xr2:uid="{183DE6D2-7FE4-EA4F-8A21-BAAE338FD231}"/>
   </bookViews>
   <sheets>
     <sheet name="Setup" sheetId="3" r:id="rId1"/>

</xml_diff>